<commit_message>
auto: actualizar indicadores adelantados 2026-06-22
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/transporte/flujo_ferroviario_1999_2026.xlsx
+++ b/datos/indicadores_adelantados/transporte/flujo_ferroviario_1999_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\1. Página Web\2026 - 05. Mayo\Transporte 03-26\Año referencial 2017\Estadisticas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\11. Otros\TRANS AGQ\Cuadros de salida Transporte\Pagina web\Estadisticas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E223AB3-F74C-4098-B146-43A8237D09E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4A87F4-DB1E-40A4-96E2-6BE09FA5F068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="27">
   <si>
     <t>PERIODO</t>
   </si>
@@ -507,7 +507,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -575,9 +575,6 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -990,7 +987,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:U396"/>
+  <dimension ref="B1:U397"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.7109375" style="2" customWidth="1"/>
@@ -1516,22 +1513,22 @@
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="2:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="32" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="29" t="s">
+      <c r="B3" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="30"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="29" t="s">
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="31"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="30"/>
     </row>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="33"/>
+      <c r="B4" s="32"/>
       <c r="C4" s="7" t="s">
         <v>22</v>
       </c>
@@ -9590,12 +9587,12 @@
       <c r="H370" s="16">
         <v>468.9</v>
       </c>
-      <c r="P370" s="28"/>
-      <c r="Q370" s="28"/>
-      <c r="R370" s="28"/>
-      <c r="S370" s="28"/>
-      <c r="T370" s="28"/>
-      <c r="U370" s="28"/>
+      <c r="P370" s="27"/>
+      <c r="Q370" s="27"/>
+      <c r="R370" s="27"/>
+      <c r="S370" s="27"/>
+      <c r="T370" s="27"/>
+      <c r="U370" s="27"/>
     </row>
     <row r="371" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B371" s="26" t="s">
@@ -9619,12 +9616,12 @@
       <c r="H371" s="15">
         <v>39.469999999999992</v>
       </c>
-      <c r="P371" s="28"/>
-      <c r="Q371" s="28"/>
-      <c r="R371" s="28"/>
-      <c r="S371" s="28"/>
-      <c r="T371" s="28"/>
-      <c r="U371" s="28"/>
+      <c r="P371" s="27"/>
+      <c r="Q371" s="27"/>
+      <c r="R371" s="27"/>
+      <c r="S371" s="27"/>
+      <c r="T371" s="27"/>
+      <c r="U371" s="27"/>
     </row>
     <row r="372" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B372" s="26" t="s">
@@ -9648,12 +9645,12 @@
       <c r="H372" s="15">
         <v>40.15</v>
       </c>
-      <c r="P372" s="28"/>
-      <c r="Q372" s="28"/>
-      <c r="R372" s="28"/>
-      <c r="S372" s="28"/>
-      <c r="T372" s="28"/>
-      <c r="U372" s="28"/>
+      <c r="P372" s="27"/>
+      <c r="Q372" s="27"/>
+      <c r="R372" s="27"/>
+      <c r="S372" s="27"/>
+      <c r="T372" s="27"/>
+      <c r="U372" s="27"/>
     </row>
     <row r="373" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B373" s="26" t="s">
@@ -9677,12 +9674,12 @@
       <c r="H373" s="15">
         <v>29.830000000000002</v>
       </c>
-      <c r="P373" s="28"/>
-      <c r="Q373" s="28"/>
-      <c r="R373" s="28"/>
-      <c r="S373" s="28"/>
-      <c r="T373" s="28"/>
-      <c r="U373" s="28"/>
+      <c r="P373" s="27"/>
+      <c r="Q373" s="27"/>
+      <c r="R373" s="27"/>
+      <c r="S373" s="27"/>
+      <c r="T373" s="27"/>
+      <c r="U373" s="27"/>
     </row>
     <row r="374" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B374" s="26" t="s">
@@ -9706,12 +9703,12 @@
       <c r="H374" s="15">
         <v>35.11</v>
       </c>
-      <c r="P374" s="28"/>
-      <c r="Q374" s="28"/>
-      <c r="R374" s="28"/>
-      <c r="S374" s="28"/>
-      <c r="T374" s="28"/>
-      <c r="U374" s="28"/>
+      <c r="P374" s="27"/>
+      <c r="Q374" s="27"/>
+      <c r="R374" s="27"/>
+      <c r="S374" s="27"/>
+      <c r="T374" s="27"/>
+      <c r="U374" s="27"/>
     </row>
     <row r="375" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B375" s="26" t="s">
@@ -9735,12 +9732,12 @@
       <c r="H375" s="15">
         <v>47.53</v>
       </c>
-      <c r="P375" s="28"/>
-      <c r="Q375" s="28"/>
-      <c r="R375" s="28"/>
-      <c r="S375" s="28"/>
-      <c r="T375" s="28"/>
-      <c r="U375" s="28"/>
+      <c r="P375" s="27"/>
+      <c r="Q375" s="27"/>
+      <c r="R375" s="27"/>
+      <c r="S375" s="27"/>
+      <c r="T375" s="27"/>
+      <c r="U375" s="27"/>
     </row>
     <row r="376" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B376" s="26" t="s">
@@ -9764,12 +9761,12 @@
       <c r="H376" s="15">
         <v>40.01</v>
       </c>
-      <c r="P376" s="28"/>
-      <c r="Q376" s="28"/>
-      <c r="R376" s="28"/>
-      <c r="S376" s="28"/>
-      <c r="T376" s="28"/>
-      <c r="U376" s="28"/>
+      <c r="P376" s="27"/>
+      <c r="Q376" s="27"/>
+      <c r="R376" s="27"/>
+      <c r="S376" s="27"/>
+      <c r="T376" s="27"/>
+      <c r="U376" s="27"/>
     </row>
     <row r="377" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B377" s="26" t="s">
@@ -9793,12 +9790,12 @@
       <c r="H377" s="15">
         <v>36.689999999999991</v>
       </c>
-      <c r="P377" s="28"/>
-      <c r="Q377" s="28"/>
-      <c r="R377" s="28"/>
-      <c r="S377" s="28"/>
-      <c r="T377" s="28"/>
-      <c r="U377" s="28"/>
+      <c r="P377" s="27"/>
+      <c r="Q377" s="27"/>
+      <c r="R377" s="27"/>
+      <c r="S377" s="27"/>
+      <c r="T377" s="27"/>
+      <c r="U377" s="27"/>
     </row>
     <row r="378" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B378" s="26" t="s">
@@ -9822,12 +9819,12 @@
       <c r="H378" s="15">
         <v>49.660000000000004</v>
       </c>
-      <c r="P378" s="28"/>
-      <c r="Q378" s="28"/>
-      <c r="R378" s="28"/>
-      <c r="S378" s="28"/>
-      <c r="T378" s="28"/>
-      <c r="U378" s="28"/>
+      <c r="P378" s="27"/>
+      <c r="Q378" s="27"/>
+      <c r="R378" s="27"/>
+      <c r="S378" s="27"/>
+      <c r="T378" s="27"/>
+      <c r="U378" s="27"/>
     </row>
     <row r="379" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B379" s="26" t="s">
@@ -9851,12 +9848,12 @@
       <c r="H379" s="15">
         <v>32.43</v>
       </c>
-      <c r="P379" s="28"/>
-      <c r="Q379" s="28"/>
-      <c r="R379" s="28"/>
-      <c r="S379" s="28"/>
-      <c r="T379" s="28"/>
-      <c r="U379" s="28"/>
+      <c r="P379" s="27"/>
+      <c r="Q379" s="27"/>
+      <c r="R379" s="27"/>
+      <c r="S379" s="27"/>
+      <c r="T379" s="27"/>
+      <c r="U379" s="27"/>
     </row>
     <row r="380" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B380" s="26" t="s">
@@ -9880,12 +9877,12 @@
       <c r="H380" s="15">
         <v>40.51</v>
       </c>
-      <c r="P380" s="28"/>
-      <c r="Q380" s="28"/>
-      <c r="R380" s="28"/>
-      <c r="S380" s="28"/>
-      <c r="T380" s="28"/>
-      <c r="U380" s="28"/>
+      <c r="P380" s="27"/>
+      <c r="Q380" s="27"/>
+      <c r="R380" s="27"/>
+      <c r="S380" s="27"/>
+      <c r="T380" s="27"/>
+      <c r="U380" s="27"/>
     </row>
     <row r="381" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B381" s="26" t="s">
@@ -9909,12 +9906,12 @@
       <c r="H381" s="15">
         <v>35.279999999999994</v>
       </c>
-      <c r="P381" s="28"/>
-      <c r="Q381" s="28"/>
-      <c r="R381" s="28"/>
-      <c r="S381" s="28"/>
-      <c r="T381" s="28"/>
-      <c r="U381" s="28"/>
+      <c r="P381" s="27"/>
+      <c r="Q381" s="27"/>
+      <c r="R381" s="27"/>
+      <c r="S381" s="27"/>
+      <c r="T381" s="27"/>
+      <c r="U381" s="27"/>
     </row>
     <row r="382" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B382" s="26" t="s">
@@ -9938,12 +9935,12 @@
       <c r="H382" s="15">
         <v>42.23</v>
       </c>
-      <c r="P382" s="28"/>
-      <c r="Q382" s="28"/>
-      <c r="R382" s="28"/>
-      <c r="S382" s="28"/>
-      <c r="T382" s="28"/>
-      <c r="U382" s="28"/>
+      <c r="P382" s="27"/>
+      <c r="Q382" s="27"/>
+      <c r="R382" s="27"/>
+      <c r="S382" s="27"/>
+      <c r="T382" s="27"/>
+      <c r="U382" s="27"/>
     </row>
     <row r="383" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B383" s="26"/>
@@ -9953,41 +9950,41 @@
       <c r="F383" s="21"/>
       <c r="G383" s="21"/>
       <c r="H383" s="15"/>
-      <c r="P383" s="28"/>
-      <c r="Q383" s="28"/>
-      <c r="R383" s="28"/>
-      <c r="S383" s="28"/>
-      <c r="T383" s="28"/>
-      <c r="U383" s="28"/>
+      <c r="P383" s="27"/>
+      <c r="Q383" s="27"/>
+      <c r="R383" s="27"/>
+      <c r="S383" s="27"/>
+      <c r="T383" s="27"/>
+      <c r="U383" s="27"/>
     </row>
     <row r="384" spans="2:21" ht="13.5" x14ac:dyDescent="0.2">
       <c r="B384" s="25" t="s">
         <v>26</v>
       </c>
       <c r="C384" s="22">
-        <v>3364</v>
+        <v>3799</v>
       </c>
       <c r="D384" s="22">
-        <v>196979.87400000001</v>
+        <v>264211.304</v>
       </c>
       <c r="E384" s="22">
         <v>0</v>
       </c>
       <c r="F384" s="22">
-        <v>768</v>
+        <v>1086</v>
       </c>
       <c r="G384" s="22">
-        <v>362762.1</v>
+        <v>509267.18000000005</v>
       </c>
       <c r="H384" s="16">
-        <v>83.92</v>
-      </c>
-      <c r="P384" s="28"/>
-      <c r="Q384" s="28"/>
-      <c r="R384" s="28"/>
-      <c r="S384" s="28"/>
-      <c r="T384" s="28"/>
-      <c r="U384" s="28"/>
+        <v>127.00999999999999</v>
+      </c>
+      <c r="P384" s="27"/>
+      <c r="Q384" s="27"/>
+      <c r="R384" s="27"/>
+      <c r="S384" s="27"/>
+      <c r="T384" s="27"/>
+      <c r="U384" s="27"/>
     </row>
     <row r="385" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B385" s="26" t="s">
@@ -10006,17 +10003,17 @@
         <v>435</v>
       </c>
       <c r="G385" s="21">
-        <v>127975.68000000001</v>
+        <v>127975.68000000002</v>
       </c>
       <c r="H385" s="15">
         <v>45.550000000000004</v>
       </c>
-      <c r="P385" s="28"/>
-      <c r="Q385" s="28"/>
-      <c r="R385" s="28"/>
-      <c r="S385" s="28"/>
-      <c r="T385" s="28"/>
-      <c r="U385" s="28"/>
+      <c r="P385" s="27"/>
+      <c r="Q385" s="27"/>
+      <c r="R385" s="27"/>
+      <c r="S385" s="27"/>
+      <c r="T385" s="27"/>
+      <c r="U385" s="27"/>
     </row>
     <row r="386" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B386" s="26" t="s">
@@ -10035,17 +10032,17 @@
         <v>38</v>
       </c>
       <c r="G386" s="21">
-        <v>101340.75</v>
+        <v>101340.75000000001</v>
       </c>
       <c r="H386" s="15">
         <v>18.61</v>
       </c>
-      <c r="P386" s="28"/>
-      <c r="Q386" s="28"/>
-      <c r="R386" s="28"/>
-      <c r="S386" s="28"/>
-      <c r="T386" s="28"/>
-      <c r="U386" s="28"/>
+      <c r="P386" s="27"/>
+      <c r="Q386" s="27"/>
+      <c r="R386" s="27"/>
+      <c r="S386" s="27"/>
+      <c r="T386" s="27"/>
+      <c r="U386" s="27"/>
     </row>
     <row r="387" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B387" s="26" t="s">
@@ -10064,78 +10061,107 @@
         <v>295</v>
       </c>
       <c r="G387" s="21">
-        <v>133445.67000000001</v>
+        <v>133445.66999999998</v>
       </c>
       <c r="H387" s="15">
         <v>19.760000000000002</v>
       </c>
-      <c r="P387" s="28"/>
-      <c r="Q387" s="28"/>
-      <c r="R387" s="28"/>
-      <c r="S387" s="28"/>
-      <c r="T387" s="28"/>
-      <c r="U387" s="28"/>
+      <c r="P387" s="27"/>
+      <c r="Q387" s="27"/>
+      <c r="R387" s="27"/>
+      <c r="S387" s="27"/>
+      <c r="T387" s="27"/>
+      <c r="U387" s="27"/>
     </row>
     <row r="388" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B388" s="27"/>
-      <c r="C388" s="23"/>
-      <c r="D388" s="23"/>
-      <c r="E388" s="24"/>
-      <c r="F388" s="23"/>
-      <c r="G388" s="23"/>
-      <c r="H388" s="24"/>
-      <c r="P388" s="28"/>
-      <c r="Q388" s="28"/>
-      <c r="R388" s="28"/>
-      <c r="S388" s="28"/>
-      <c r="T388" s="28"/>
-      <c r="U388" s="28"/>
-    </row>
-    <row r="389" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B389" s="19" t="s">
+      <c r="B388" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C388" s="21">
+        <v>435</v>
+      </c>
+      <c r="D388" s="21">
+        <v>67231.429999999978</v>
+      </c>
+      <c r="E388" s="15">
+        <v>0</v>
+      </c>
+      <c r="F388" s="21">
+        <v>318</v>
+      </c>
+      <c r="G388" s="21">
+        <v>146505.07999999999</v>
+      </c>
+      <c r="H388" s="15">
+        <v>43.089999999999996</v>
+      </c>
+      <c r="P388" s="27"/>
+      <c r="Q388" s="27"/>
+      <c r="R388" s="27"/>
+      <c r="S388" s="27"/>
+      <c r="T388" s="27"/>
+      <c r="U388" s="27"/>
+    </row>
+    <row r="389" spans="2:21" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B389" s="26"/>
+      <c r="C389" s="23"/>
+      <c r="D389" s="23"/>
+      <c r="E389" s="24"/>
+      <c r="F389" s="23"/>
+      <c r="G389" s="23"/>
+      <c r="H389" s="24"/>
+      <c r="P389" s="27"/>
+      <c r="Q389" s="27"/>
+      <c r="R389" s="27"/>
+      <c r="S389" s="27"/>
+      <c r="T389" s="27"/>
+      <c r="U389" s="27"/>
+    </row>
+    <row r="390" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B390" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C389" s="18"/>
-      <c r="D389" s="18"/>
-      <c r="E389" s="18"/>
-      <c r="F389" s="18"/>
-      <c r="G389" s="18"/>
-      <c r="H389" s="18"/>
-    </row>
-    <row r="390" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B390" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C390" s="11"/>
+      <c r="C390" s="18"/>
+      <c r="D390" s="18"/>
+      <c r="E390" s="18"/>
+      <c r="F390" s="18"/>
+      <c r="G390" s="18"/>
+      <c r="H390" s="18"/>
     </row>
     <row r="391" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B391" s="20" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C391" s="11"/>
-      <c r="H391" s="5"/>
     </row>
     <row r="392" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B392" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C392" s="11"/>
+      <c r="H392" s="5"/>
+    </row>
+    <row r="393" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B393" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C392" s="11"/>
-    </row>
-    <row r="393" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B393" s="17"/>
       <c r="C393" s="11"/>
     </row>
     <row r="394" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B394" s="17"/>
-      <c r="C394" s="14"/>
+      <c r="C394" s="11"/>
     </row>
     <row r="395" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B395" s="12"/>
+      <c r="B395" s="17"/>
       <c r="C395" s="14"/>
     </row>
     <row r="396" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B396" s="12"/>
-      <c r="C396" s="13"/>
+      <c r="C396" s="14"/>
+    </row>
+    <row r="397" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B397" s="12"/>
+      <c r="C397" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>